<commit_message>
feat: add JAX frequency score and Markov sequence probability calculation for the last combination
</commit_message>
<xml_diff>
--- a/baloto.xlsx
+++ b/baloto.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Baloto" sheetId="1" state="visible" r:id="rId3"/>
@@ -259,7 +259,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -380,10 +380,6 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -405,7 +401,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -417,14 +413,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F1F1F"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -26890,7 +26878,7 @@
         <v>10</v>
       </c>
       <c r="H903" s="3" t="n">
-        <v>29000000</v>
+        <v>290000000</v>
       </c>
       <c r="I903" s="3" t="n">
         <v>0</v>
@@ -30133,7 +30121,7 @@
       <c r="I49" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="O49" s="30"/>
+      <c r="O49" s="25"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="27" t="n">
@@ -30165,7 +30153,7 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="31" t="n">
+      <c r="A51" s="30" t="n">
         <v>43019</v>
       </c>
       <c r="B51" s="28" t="n">
@@ -30194,7 +30182,7 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="31" t="n">
+      <c r="A52" s="30" t="n">
         <v>43022</v>
       </c>
       <c r="B52" s="28" t="n">
@@ -30223,7 +30211,7 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="31" t="n">
+      <c r="A53" s="30" t="n">
         <v>43026</v>
       </c>
       <c r="B53" s="28" t="n">
@@ -30252,7 +30240,7 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="31" t="n">
+      <c r="A54" s="30" t="n">
         <v>43029</v>
       </c>
       <c r="B54" s="28" t="n">
@@ -30281,7 +30269,7 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="31" t="n">
+      <c r="A55" s="30" t="n">
         <v>43033</v>
       </c>
       <c r="B55" s="28" t="n">
@@ -30310,7 +30298,7 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="31" t="n">
+      <c r="A56" s="30" t="n">
         <v>43036</v>
       </c>
       <c r="B56" s="28" t="n">
@@ -30426,7 +30414,7 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="31" t="n">
+      <c r="A60" s="30" t="n">
         <v>43050</v>
       </c>
       <c r="B60" s="28" t="n">
@@ -30455,7 +30443,7 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="31" t="n">
+      <c r="A61" s="30" t="n">
         <v>43054</v>
       </c>
       <c r="B61" s="28" t="n">
@@ -30484,7 +30472,7 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="31" t="n">
+      <c r="A62" s="30" t="n">
         <v>43057</v>
       </c>
       <c r="B62" s="28" t="n">
@@ -30513,7 +30501,7 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="31" t="n">
+      <c r="A63" s="30" t="n">
         <v>43061</v>
       </c>
       <c r="B63" s="28" t="n">
@@ -30542,7 +30530,7 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="31" t="n">
+      <c r="A64" s="30" t="n">
         <v>43064</v>
       </c>
       <c r="B64" s="28" t="n">
@@ -30571,7 +30559,7 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="31" t="n">
+      <c r="A65" s="30" t="n">
         <v>43068</v>
       </c>
       <c r="B65" s="28" t="n">
@@ -30687,7 +30675,7 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="31" t="n">
+      <c r="A69" s="30" t="n">
         <v>43082</v>
       </c>
       <c r="B69" s="28" t="n">
@@ -30716,7 +30704,7 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="31" t="n">
+      <c r="A70" s="30" t="n">
         <v>43085</v>
       </c>
       <c r="B70" s="28" t="n">
@@ -30745,7 +30733,7 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="31" t="n">
+      <c r="A71" s="30" t="n">
         <v>43089</v>
       </c>
       <c r="B71" s="28" t="n">
@@ -30774,7 +30762,7 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="31" t="n">
+      <c r="A72" s="30" t="n">
         <v>43092</v>
       </c>
       <c r="B72" s="28" t="n">
@@ -30803,7 +30791,7 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="31" t="n">
+      <c r="A73" s="30" t="n">
         <v>43096</v>
       </c>
       <c r="B73" s="28" t="n">
@@ -30832,7 +30820,7 @@
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="31" t="n">
+      <c r="A74" s="30" t="n">
         <v>43099</v>
       </c>
       <c r="B74" s="28" t="n">
@@ -33181,7 +33169,7 @@
       </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="31" t="n">
+      <c r="A155" s="30" t="n">
         <v>43383</v>
       </c>
       <c r="B155" s="28" t="n">
@@ -33210,7 +33198,7 @@
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A156" s="31" t="n">
+      <c r="A156" s="30" t="n">
         <v>43386</v>
       </c>
       <c r="B156" s="28" t="n">
@@ -33239,7 +33227,7 @@
       </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="31" t="n">
+      <c r="A157" s="30" t="n">
         <v>43390</v>
       </c>
       <c r="B157" s="28" t="n">
@@ -33268,7 +33256,7 @@
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A158" s="31" t="n">
+      <c r="A158" s="30" t="n">
         <v>43393</v>
       </c>
       <c r="B158" s="28" t="n">
@@ -33297,7 +33285,7 @@
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A159" s="31" t="n">
+      <c r="A159" s="30" t="n">
         <v>43397</v>
       </c>
       <c r="B159" s="28" t="n">
@@ -33326,7 +33314,7 @@
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="31" t="n">
+      <c r="A160" s="30" t="n">
         <v>43400</v>
       </c>
       <c r="B160" s="28" t="n">
@@ -33355,7 +33343,7 @@
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="31" t="n">
+      <c r="A161" s="30" t="n">
         <v>43404</v>
       </c>
       <c r="B161" s="28" t="n">
@@ -33442,7 +33430,7 @@
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="31" t="n">
+      <c r="A164" s="30" t="n">
         <v>43414</v>
       </c>
       <c r="B164" s="28" t="n">
@@ -33471,7 +33459,7 @@
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="31" t="n">
+      <c r="A165" s="30" t="n">
         <v>43418</v>
       </c>
       <c r="B165" s="28" t="n">
@@ -33500,7 +33488,7 @@
       </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A166" s="31" t="n">
+      <c r="A166" s="30" t="n">
         <v>43421</v>
       </c>
       <c r="B166" s="28" t="n">
@@ -33529,7 +33517,7 @@
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="31" t="n">
+      <c r="A167" s="30" t="n">
         <v>43425</v>
       </c>
       <c r="B167" s="28" t="n">
@@ -33558,7 +33546,7 @@
       </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="31" t="n">
+      <c r="A168" s="30" t="n">
         <v>43428</v>
       </c>
       <c r="B168" s="28" t="n">
@@ -33587,7 +33575,7 @@
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A169" s="31" t="n">
+      <c r="A169" s="30" t="n">
         <v>43432</v>
       </c>
       <c r="B169" s="28" t="n">
@@ -33703,7 +33691,7 @@
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A173" s="31" t="n">
+      <c r="A173" s="30" t="n">
         <v>43446</v>
       </c>
       <c r="B173" s="28" t="n">
@@ -33732,7 +33720,7 @@
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A174" s="31" t="n">
+      <c r="A174" s="30" t="n">
         <v>43449</v>
       </c>
       <c r="B174" s="28" t="n">
@@ -33761,7 +33749,7 @@
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A175" s="31" t="n">
+      <c r="A175" s="30" t="n">
         <v>43453</v>
       </c>
       <c r="B175" s="28" t="n">
@@ -33790,7 +33778,7 @@
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="31" t="n">
+      <c r="A176" s="30" t="n">
         <v>43456</v>
       </c>
       <c r="B176" s="28" t="n">
@@ -33819,7 +33807,7 @@
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="31" t="n">
+      <c r="A177" s="30" t="n">
         <v>43460</v>
       </c>
       <c r="B177" s="28" t="n">
@@ -33848,7 +33836,7 @@
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="31" t="n">
+      <c r="A178" s="30" t="n">
         <v>43463</v>
       </c>
       <c r="B178" s="28" t="n">
@@ -36226,7 +36214,7 @@
       </c>
     </row>
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A260" s="31" t="n">
+      <c r="A260" s="30" t="n">
         <v>43750</v>
       </c>
       <c r="B260" s="28" t="n">
@@ -36255,7 +36243,7 @@
       </c>
     </row>
     <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A261" s="31" t="n">
+      <c r="A261" s="30" t="n">
         <v>43754</v>
       </c>
       <c r="B261" s="28" t="n">
@@ -36284,7 +36272,7 @@
       </c>
     </row>
     <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A262" s="31" t="n">
+      <c r="A262" s="30" t="n">
         <v>43757</v>
       </c>
       <c r="B262" s="28" t="n">
@@ -36313,7 +36301,7 @@
       </c>
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A263" s="31" t="n">
+      <c r="A263" s="30" t="n">
         <v>43761</v>
       </c>
       <c r="B263" s="28" t="n">
@@ -36342,7 +36330,7 @@
       </c>
     </row>
     <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A264" s="31" t="n">
+      <c r="A264" s="30" t="n">
         <v>43764</v>
       </c>
       <c r="B264" s="28" t="n">
@@ -36371,7 +36359,7 @@
       </c>
     </row>
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A265" s="31" t="n">
+      <c r="A265" s="30" t="n">
         <v>43768</v>
       </c>
       <c r="B265" s="28" t="n">
@@ -36487,7 +36475,7 @@
       </c>
     </row>
     <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A269" s="31" t="n">
+      <c r="A269" s="30" t="n">
         <v>43782</v>
       </c>
       <c r="B269" s="28" t="n">
@@ -36516,7 +36504,7 @@
       </c>
     </row>
     <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A270" s="31" t="n">
+      <c r="A270" s="30" t="n">
         <v>43785</v>
       </c>
       <c r="B270" s="28" t="n">
@@ -36545,7 +36533,7 @@
       </c>
     </row>
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A271" s="31" t="n">
+      <c r="A271" s="30" t="n">
         <v>43789</v>
       </c>
       <c r="B271" s="28" t="n">
@@ -36574,7 +36562,7 @@
       </c>
     </row>
     <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A272" s="31" t="n">
+      <c r="A272" s="30" t="n">
         <v>43792</v>
       </c>
       <c r="B272" s="28" t="n">
@@ -36603,7 +36591,7 @@
       </c>
     </row>
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A273" s="31" t="n">
+      <c r="A273" s="30" t="n">
         <v>43796</v>
       </c>
       <c r="B273" s="28" t="n">
@@ -36632,7 +36620,7 @@
       </c>
     </row>
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A274" s="31" t="n">
+      <c r="A274" s="30" t="n">
         <v>43799</v>
       </c>
       <c r="B274" s="28" t="n">
@@ -36719,7 +36707,7 @@
       </c>
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A277" s="31" t="n">
+      <c r="A277" s="30" t="n">
         <v>43810</v>
       </c>
       <c r="B277" s="28" t="n">
@@ -36748,7 +36736,7 @@
       </c>
     </row>
     <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A278" s="31" t="n">
+      <c r="A278" s="30" t="n">
         <v>43813</v>
       </c>
       <c r="B278" s="28" t="n">
@@ -36777,7 +36765,7 @@
       </c>
     </row>
     <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A279" s="31" t="n">
+      <c r="A279" s="30" t="n">
         <v>43817</v>
       </c>
       <c r="B279" s="28" t="n">
@@ -36806,7 +36794,7 @@
       </c>
     </row>
     <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A280" s="31" t="n">
+      <c r="A280" s="30" t="n">
         <v>43820</v>
       </c>
       <c r="B280" s="28" t="n">
@@ -36835,7 +36823,7 @@
       </c>
     </row>
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A281" s="31" t="n">
+      <c r="A281" s="30" t="n">
         <v>43824</v>
       </c>
       <c r="B281" s="28" t="n">
@@ -36864,7 +36852,7 @@
       </c>
     </row>
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A282" s="31" t="n">
+      <c r="A282" s="30" t="n">
         <v>43827</v>
       </c>
       <c r="B282" s="28" t="n">
@@ -38952,7 +38940,7 @@
       </c>
     </row>
     <row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A354" s="31" t="n">
+      <c r="A354" s="30" t="n">
         <v>44114</v>
       </c>
       <c r="B354" s="28" t="n">
@@ -38981,7 +38969,7 @@
       </c>
     </row>
     <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A355" s="31" t="n">
+      <c r="A355" s="30" t="n">
         <v>44118</v>
       </c>
       <c r="B355" s="28" t="n">
@@ -39010,7 +38998,7 @@
       </c>
     </row>
     <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A356" s="31" t="n">
+      <c r="A356" s="30" t="n">
         <v>44121</v>
       </c>
       <c r="B356" s="28" t="n">
@@ -39039,7 +39027,7 @@
       </c>
     </row>
     <row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A357" s="31" t="n">
+      <c r="A357" s="30" t="n">
         <v>44125</v>
       </c>
       <c r="B357" s="28" t="n">
@@ -39068,7 +39056,7 @@
       </c>
     </row>
     <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A358" s="31" t="n">
+      <c r="A358" s="30" t="n">
         <v>44128</v>
       </c>
       <c r="B358" s="28" t="n">
@@ -39097,7 +39085,7 @@
       </c>
     </row>
     <row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A359" s="31" t="n">
+      <c r="A359" s="30" t="n">
         <v>44132</v>
       </c>
       <c r="B359" s="28" t="n">
@@ -39126,7 +39114,7 @@
       </c>
     </row>
     <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A360" s="31" t="n">
+      <c r="A360" s="30" t="n">
         <v>44135</v>
       </c>
       <c r="B360" s="28" t="n">
@@ -39213,7 +39201,7 @@
       </c>
     </row>
     <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A363" s="31" t="n">
+      <c r="A363" s="30" t="n">
         <v>44146</v>
       </c>
       <c r="B363" s="28" t="n">
@@ -39242,7 +39230,7 @@
       </c>
     </row>
     <row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A364" s="31" t="n">
+      <c r="A364" s="30" t="n">
         <v>44149</v>
       </c>
       <c r="B364" s="28" t="n">
@@ -39271,7 +39259,7 @@
       </c>
     </row>
     <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A365" s="31" t="n">
+      <c r="A365" s="30" t="n">
         <v>44153</v>
       </c>
       <c r="B365" s="28" t="n">
@@ -39300,7 +39288,7 @@
       </c>
     </row>
     <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A366" s="31" t="n">
+      <c r="A366" s="30" t="n">
         <v>44156</v>
       </c>
       <c r="B366" s="28" t="n">
@@ -39329,7 +39317,7 @@
       </c>
     </row>
     <row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A367" s="31" t="n">
+      <c r="A367" s="30" t="n">
         <v>44160</v>
       </c>
       <c r="B367" s="28" t="n">
@@ -39358,7 +39346,7 @@
       </c>
     </row>
     <row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A368" s="31" t="n">
+      <c r="A368" s="30" t="n">
         <v>44163</v>
       </c>
       <c r="B368" s="28" t="n">
@@ -39474,7 +39462,7 @@
       </c>
     </row>
     <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A372" s="31" t="n">
+      <c r="A372" s="30" t="n">
         <v>44177</v>
       </c>
       <c r="B372" s="28" t="n">
@@ -39503,7 +39491,7 @@
       </c>
     </row>
     <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A373" s="31" t="n">
+      <c r="A373" s="30" t="n">
         <v>44181</v>
       </c>
       <c r="B373" s="28" t="n">
@@ -39532,7 +39520,7 @@
       </c>
     </row>
     <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A374" s="31" t="n">
+      <c r="A374" s="30" t="n">
         <v>44184</v>
       </c>
       <c r="B374" s="28" t="n">
@@ -39561,7 +39549,7 @@
       </c>
     </row>
     <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A375" s="31" t="n">
+      <c r="A375" s="30" t="n">
         <v>44188</v>
       </c>
       <c r="B375" s="28" t="n">
@@ -39590,7 +39578,7 @@
       </c>
     </row>
     <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A376" s="31" t="n">
+      <c r="A376" s="30" t="n">
         <v>44191</v>
       </c>
       <c r="B376" s="28" t="n">
@@ -39619,7 +39607,7 @@
       </c>
     </row>
     <row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A377" s="31" t="n">
+      <c r="A377" s="30" t="n">
         <v>44195</v>
       </c>
       <c r="B377" s="28" t="n">
@@ -41997,7 +41985,7 @@
       </c>
     </row>
     <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A459" s="31" t="n">
+      <c r="A459" s="30" t="n">
         <v>44482</v>
       </c>
       <c r="B459" s="28" t="n">
@@ -42026,7 +42014,7 @@
       </c>
     </row>
     <row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A460" s="31" t="n">
+      <c r="A460" s="30" t="n">
         <v>44485</v>
       </c>
       <c r="B460" s="28" t="n">
@@ -42055,7 +42043,7 @@
       </c>
     </row>
     <row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A461" s="31" t="n">
+      <c r="A461" s="30" t="n">
         <v>44489</v>
       </c>
       <c r="B461" s="28" t="n">
@@ -42084,7 +42072,7 @@
       </c>
     </row>
     <row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A462" s="31" t="n">
+      <c r="A462" s="30" t="n">
         <v>44492</v>
       </c>
       <c r="B462" s="28" t="n">
@@ -42113,7 +42101,7 @@
       </c>
     </row>
     <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A463" s="31" t="n">
+      <c r="A463" s="30" t="n">
         <v>44496</v>
       </c>
       <c r="B463" s="28" t="n">
@@ -42142,7 +42130,7 @@
       </c>
     </row>
     <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A464" s="31" t="n">
+      <c r="A464" s="30" t="n">
         <v>44499</v>
       </c>
       <c r="B464" s="28" t="n">
@@ -42229,7 +42217,7 @@
       </c>
     </row>
     <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A467" s="31" t="n">
+      <c r="A467" s="30" t="n">
         <v>44510</v>
       </c>
       <c r="B467" s="28" t="n">
@@ -42258,7 +42246,7 @@
       </c>
     </row>
     <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A468" s="31" t="n">
+      <c r="A468" s="30" t="n">
         <v>44513</v>
       </c>
       <c r="B468" s="28" t="n">
@@ -42287,7 +42275,7 @@
       </c>
     </row>
     <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A469" s="31" t="n">
+      <c r="A469" s="30" t="n">
         <v>44517</v>
       </c>
       <c r="B469" s="28" t="n">
@@ -42316,7 +42304,7 @@
       </c>
     </row>
     <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A470" s="31" t="n">
+      <c r="A470" s="30" t="n">
         <v>44520</v>
       </c>
       <c r="B470" s="28" t="n">
@@ -42345,7 +42333,7 @@
       </c>
     </row>
     <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A471" s="31" t="n">
+      <c r="A471" s="30" t="n">
         <v>44524</v>
       </c>
       <c r="B471" s="28" t="n">
@@ -42374,7 +42362,7 @@
       </c>
     </row>
     <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A472" s="31" t="n">
+      <c r="A472" s="30" t="n">
         <v>44527</v>
       </c>
       <c r="B472" s="28" t="n">
@@ -42490,7 +42478,7 @@
       </c>
     </row>
     <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A476" s="31" t="n">
+      <c r="A476" s="30" t="n">
         <v>44541</v>
       </c>
       <c r="B476" s="28" t="n">
@@ -42519,7 +42507,7 @@
       </c>
     </row>
     <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A477" s="31" t="n">
+      <c r="A477" s="30" t="n">
         <v>44545</v>
       </c>
       <c r="B477" s="28" t="n">
@@ -42548,7 +42536,7 @@
       </c>
     </row>
     <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A478" s="31" t="n">
+      <c r="A478" s="30" t="n">
         <v>44548</v>
       </c>
       <c r="B478" s="28" t="n">
@@ -42577,7 +42565,7 @@
       </c>
     </row>
     <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A479" s="31" t="n">
+      <c r="A479" s="30" t="n">
         <v>44552</v>
       </c>
       <c r="B479" s="28" t="n">
@@ -42606,7 +42594,7 @@
       </c>
     </row>
     <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A480" s="31" t="n">
+      <c r="A480" s="30" t="n">
         <v>44555</v>
       </c>
       <c r="B480" s="28" t="n">
@@ -42635,7 +42623,7 @@
       </c>
     </row>
     <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A481" s="31" t="n">
+      <c r="A481" s="30" t="n">
         <v>44559</v>
       </c>
       <c r="B481" s="28" t="n">
@@ -45013,7 +45001,7 @@
       </c>
     </row>
     <row r="563" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A563" s="31" t="n">
+      <c r="A563" s="30" t="n">
         <v>44846</v>
       </c>
       <c r="B563" s="28" t="n">
@@ -45042,7 +45030,7 @@
       </c>
     </row>
     <row r="564" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A564" s="31" t="n">
+      <c r="A564" s="30" t="n">
         <v>44849</v>
       </c>
       <c r="B564" s="28" t="n">
@@ -45071,7 +45059,7 @@
       </c>
     </row>
     <row r="565" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A565" s="31" t="n">
+      <c r="A565" s="30" t="n">
         <v>44853</v>
       </c>
       <c r="B565" s="28" t="n">
@@ -45100,7 +45088,7 @@
       </c>
     </row>
     <row r="566" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A566" s="31" t="n">
+      <c r="A566" s="30" t="n">
         <v>44856</v>
       </c>
       <c r="B566" s="28" t="n">
@@ -45129,7 +45117,7 @@
       </c>
     </row>
     <row r="567" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A567" s="31" t="n">
+      <c r="A567" s="30" t="n">
         <v>44860</v>
       </c>
       <c r="B567" s="28" t="n">
@@ -45158,7 +45146,7 @@
       </c>
     </row>
     <row r="568" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A568" s="31" t="n">
+      <c r="A568" s="30" t="n">
         <v>44863</v>
       </c>
       <c r="B568" s="28" t="n">
@@ -45274,7 +45262,7 @@
       </c>
     </row>
     <row r="572" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A572" s="31" t="n">
+      <c r="A572" s="30" t="n">
         <v>44877</v>
       </c>
       <c r="B572" s="28" t="n">
@@ -45303,7 +45291,7 @@
       </c>
     </row>
     <row r="573" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A573" s="31" t="n">
+      <c r="A573" s="30" t="n">
         <v>44881</v>
       </c>
       <c r="B573" s="28" t="n">
@@ -45332,7 +45320,7 @@
       </c>
     </row>
     <row r="574" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A574" s="31" t="n">
+      <c r="A574" s="30" t="n">
         <v>44884</v>
       </c>
       <c r="B574" s="28" t="n">
@@ -45361,7 +45349,7 @@
       </c>
     </row>
     <row r="575" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A575" s="31" t="n">
+      <c r="A575" s="30" t="n">
         <v>44888</v>
       </c>
       <c r="B575" s="28" t="n">
@@ -45390,7 +45378,7 @@
       </c>
     </row>
     <row r="576" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A576" s="31" t="n">
+      <c r="A576" s="30" t="n">
         <v>44891</v>
       </c>
       <c r="B576" s="28" t="n">
@@ -45419,7 +45407,7 @@
       </c>
     </row>
     <row r="577" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A577" s="31" t="n">
+      <c r="A577" s="30" t="n">
         <v>44895</v>
       </c>
       <c r="B577" s="28" t="n">
@@ -45506,7 +45494,7 @@
       </c>
     </row>
     <row r="580" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A580" s="31" t="n">
+      <c r="A580" s="30" t="n">
         <v>44905</v>
       </c>
       <c r="B580" s="28" t="n">
@@ -45535,7 +45523,7 @@
       </c>
     </row>
     <row r="581" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A581" s="31" t="n">
+      <c r="A581" s="30" t="n">
         <v>44909</v>
       </c>
       <c r="B581" s="28" t="n">
@@ -45564,7 +45552,7 @@
       </c>
     </row>
     <row r="582" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A582" s="31" t="n">
+      <c r="A582" s="30" t="n">
         <v>44912</v>
       </c>
       <c r="B582" s="28" t="n">
@@ -45593,7 +45581,7 @@
       </c>
     </row>
     <row r="583" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A583" s="31" t="n">
+      <c r="A583" s="30" t="n">
         <v>44916</v>
       </c>
       <c r="B583" s="28" t="n">
@@ -45622,7 +45610,7 @@
       </c>
     </row>
     <row r="584" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A584" s="31" t="n">
+      <c r="A584" s="30" t="n">
         <v>44919</v>
       </c>
       <c r="B584" s="28" t="n">
@@ -45651,7 +45639,7 @@
       </c>
     </row>
     <row r="585" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A585" s="31" t="n">
+      <c r="A585" s="30" t="n">
         <v>44923</v>
       </c>
       <c r="B585" s="28" t="n">
@@ -45680,7 +45668,7 @@
       </c>
     </row>
     <row r="586" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A586" s="31" t="n">
+      <c r="A586" s="30" t="n">
         <v>44926</v>
       </c>
       <c r="B586" s="28" t="n">
@@ -48029,7 +48017,7 @@
       </c>
     </row>
     <row r="667" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A667" s="31" t="n">
+      <c r="A667" s="30" t="n">
         <v>45210</v>
       </c>
       <c r="B667" s="28" t="n">
@@ -48058,7 +48046,7 @@
       </c>
     </row>
     <row r="668" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A668" s="31" t="n">
+      <c r="A668" s="30" t="n">
         <v>45213</v>
       </c>
       <c r="B668" s="28" t="n">
@@ -48087,7 +48075,7 @@
       </c>
     </row>
     <row r="669" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A669" s="31" t="n">
+      <c r="A669" s="30" t="n">
         <v>45217</v>
       </c>
       <c r="B669" s="28" t="n">
@@ -48116,7 +48104,7 @@
       </c>
     </row>
     <row r="670" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A670" s="31" t="n">
+      <c r="A670" s="30" t="n">
         <v>45220</v>
       </c>
       <c r="B670" s="28" t="n">
@@ -48145,7 +48133,7 @@
       </c>
     </row>
     <row r="671" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A671" s="31" t="n">
+      <c r="A671" s="30" t="n">
         <v>45224</v>
       </c>
       <c r="B671" s="28" t="n">
@@ -48174,7 +48162,7 @@
       </c>
     </row>
     <row r="672" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A672" s="31" t="n">
+      <c r="A672" s="30" t="n">
         <v>45227</v>
       </c>
       <c r="B672" s="28" t="n">
@@ -48290,7 +48278,7 @@
       </c>
     </row>
     <row r="676" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A676" s="31" t="n">
+      <c r="A676" s="30" t="n">
         <v>45241</v>
       </c>
       <c r="B676" s="28" t="n">
@@ -48319,7 +48307,7 @@
       </c>
     </row>
     <row r="677" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A677" s="31" t="n">
+      <c r="A677" s="30" t="n">
         <v>45245</v>
       </c>
       <c r="B677" s="28" t="n">
@@ -48348,7 +48336,7 @@
       </c>
     </row>
     <row r="678" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A678" s="31" t="n">
+      <c r="A678" s="30" t="n">
         <v>45248</v>
       </c>
       <c r="B678" s="28" t="n">
@@ -48377,7 +48365,7 @@
       </c>
     </row>
     <row r="679" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A679" s="31" t="n">
+      <c r="A679" s="30" t="n">
         <v>45252</v>
       </c>
       <c r="B679" s="28" t="n">
@@ -48406,7 +48394,7 @@
       </c>
     </row>
     <row r="680" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A680" s="31" t="n">
+      <c r="A680" s="30" t="n">
         <v>45255</v>
       </c>
       <c r="B680" s="28" t="n">
@@ -48435,7 +48423,7 @@
       </c>
     </row>
     <row r="681" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A681" s="31" t="n">
+      <c r="A681" s="30" t="n">
         <v>45259</v>
       </c>
       <c r="B681" s="28" t="n">
@@ -48551,7 +48539,7 @@
       </c>
     </row>
     <row r="685" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A685" s="31" t="n">
+      <c r="A685" s="30" t="n">
         <v>45273</v>
       </c>
       <c r="B685" s="28" t="n">
@@ -48580,7 +48568,7 @@
       </c>
     </row>
     <row r="686" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A686" s="31" t="n">
+      <c r="A686" s="30" t="n">
         <v>45276</v>
       </c>
       <c r="B686" s="28" t="n">
@@ -48609,7 +48597,7 @@
       </c>
     </row>
     <row r="687" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A687" s="31" t="n">
+      <c r="A687" s="30" t="n">
         <v>45280</v>
       </c>
       <c r="B687" s="28" t="n">
@@ -48638,7 +48626,7 @@
       </c>
     </row>
     <row r="688" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A688" s="31" t="n">
+      <c r="A688" s="30" t="n">
         <v>45283</v>
       </c>
       <c r="B688" s="28" t="n">
@@ -48667,7 +48655,7 @@
       </c>
     </row>
     <row r="689" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A689" s="31" t="n">
+      <c r="A689" s="30" t="n">
         <v>45287</v>
       </c>
       <c r="B689" s="28" t="n">
@@ -48696,7 +48684,7 @@
       </c>
     </row>
     <row r="690" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A690" s="31" t="n">
+      <c r="A690" s="30" t="n">
         <v>45290</v>
       </c>
       <c r="B690" s="28" t="n">
@@ -51074,7 +51062,7 @@
       </c>
     </row>
     <row r="772" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A772" s="31" t="n">
+      <c r="A772" s="30" t="n">
         <v>45577</v>
       </c>
       <c r="B772" s="28" t="n">
@@ -51103,7 +51091,7 @@
       </c>
     </row>
     <row r="773" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A773" s="31" t="n">
+      <c r="A773" s="30" t="n">
         <v>45581</v>
       </c>
       <c r="B773" s="28" t="n">
@@ -51132,7 +51120,7 @@
       </c>
     </row>
     <row r="774" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A774" s="31" t="n">
+      <c r="A774" s="30" t="n">
         <v>45584</v>
       </c>
       <c r="B774" s="28" t="n">
@@ -51161,7 +51149,7 @@
       </c>
     </row>
     <row r="775" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A775" s="31" t="n">
+      <c r="A775" s="30" t="n">
         <v>45588</v>
       </c>
       <c r="B775" s="28" t="n">
@@ -51190,7 +51178,7 @@
       </c>
     </row>
     <row r="776" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A776" s="31" t="n">
+      <c r="A776" s="30" t="n">
         <v>45591</v>
       </c>
       <c r="B776" s="28" t="n">
@@ -51219,7 +51207,7 @@
       </c>
     </row>
     <row r="777" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A777" s="31" t="n">
+      <c r="A777" s="30" t="n">
         <v>45595</v>
       </c>
       <c r="B777" s="28" t="n">
@@ -51335,7 +51323,7 @@
       </c>
     </row>
     <row r="781" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A781" s="31" t="n">
+      <c r="A781" s="30" t="n">
         <v>45609</v>
       </c>
       <c r="B781" s="28" t="n">
@@ -51364,7 +51352,7 @@
       </c>
     </row>
     <row r="782" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A782" s="31" t="n">
+      <c r="A782" s="30" t="n">
         <v>45612</v>
       </c>
       <c r="B782" s="28" t="n">
@@ -51393,7 +51381,7 @@
       </c>
     </row>
     <row r="783" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A783" s="31" t="n">
+      <c r="A783" s="30" t="n">
         <v>45616</v>
       </c>
       <c r="B783" s="28" t="n">
@@ -51422,7 +51410,7 @@
       </c>
     </row>
     <row r="784" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A784" s="31" t="n">
+      <c r="A784" s="30" t="n">
         <v>45619</v>
       </c>
       <c r="B784" s="28" t="n">
@@ -51451,7 +51439,7 @@
       </c>
     </row>
     <row r="785" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A785" s="31" t="n">
+      <c r="A785" s="30" t="n">
         <v>45623</v>
       </c>
       <c r="B785" s="28" t="n">
@@ -51480,7 +51468,7 @@
       </c>
     </row>
     <row r="786" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A786" s="31" t="n">
+      <c r="A786" s="30" t="n">
         <v>45626</v>
       </c>
       <c r="B786" s="28" t="n">
@@ -51567,7 +51555,7 @@
       </c>
     </row>
     <row r="789" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A789" s="31" t="n">
+      <c r="A789" s="30" t="n">
         <v>45637</v>
       </c>
       <c r="B789" s="28" t="n">
@@ -51596,7 +51584,7 @@
       </c>
     </row>
     <row r="790" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A790" s="31" t="n">
+      <c r="A790" s="30" t="n">
         <v>45640</v>
       </c>
       <c r="B790" s="28" t="n">
@@ -51625,7 +51613,7 @@
       </c>
     </row>
     <row r="791" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A791" s="31" t="n">
+      <c r="A791" s="30" t="n">
         <v>45644</v>
       </c>
       <c r="B791" s="28" t="n">
@@ -51654,7 +51642,7 @@
       </c>
     </row>
     <row r="792" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A792" s="31" t="n">
+      <c r="A792" s="30" t="n">
         <v>45647</v>
       </c>
       <c r="B792" s="28" t="n">
@@ -51683,7 +51671,7 @@
       </c>
     </row>
     <row r="793" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A793" s="31" t="n">
+      <c r="A793" s="30" t="n">
         <v>45651</v>
       </c>
       <c r="B793" s="28" t="n">
@@ -51712,7 +51700,7 @@
       </c>
     </row>
     <row r="794" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A794" s="31" t="n">
+      <c r="A794" s="30" t="n">
         <v>45654</v>
       </c>
       <c r="B794" s="28" t="n">
@@ -51947,22 +51935,22 @@
       <c r="A802" s="27" t="n">
         <v>45682</v>
       </c>
-      <c r="B802" s="32" t="n">
+      <c r="B802" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="C802" s="33" t="n">
+      <c r="C802" s="32" t="n">
         <v>26</v>
       </c>
-      <c r="D802" s="33" t="n">
+      <c r="D802" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="E802" s="33" t="n">
+      <c r="E802" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="F802" s="33" t="n">
+      <c r="F802" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="G802" s="33" t="n">
+      <c r="G802" s="32" t="n">
         <v>5</v>
       </c>
       <c r="H802" s="12" t="n">
@@ -51976,22 +51964,22 @@
       <c r="A803" s="27" t="n">
         <v>45686</v>
       </c>
-      <c r="B803" s="32" t="n">
+      <c r="B803" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="C803" s="33" t="n">
+      <c r="C803" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="D803" s="33" t="n">
+      <c r="D803" s="32" t="n">
         <v>33</v>
       </c>
-      <c r="E803" s="33" t="n">
+      <c r="E803" s="32" t="n">
         <v>36</v>
       </c>
-      <c r="F803" s="33" t="n">
+      <c r="F803" s="32" t="n">
         <v>39</v>
       </c>
-      <c r="G803" s="33" t="n">
+      <c r="G803" s="32" t="n">
         <v>10</v>
       </c>
       <c r="H803" s="12" t="n">
@@ -52005,22 +51993,22 @@
       <c r="A804" s="27" t="n">
         <v>45689</v>
       </c>
-      <c r="B804" s="32" t="n">
+      <c r="B804" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C804" s="33" t="n">
+      <c r="C804" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="D804" s="33" t="n">
+      <c r="D804" s="32" t="n">
         <v>19</v>
       </c>
-      <c r="E804" s="33" t="n">
+      <c r="E804" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="F804" s="33" t="n">
+      <c r="F804" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="G804" s="33" t="n">
+      <c r="G804" s="32" t="n">
         <v>16</v>
       </c>
       <c r="H804" s="12" t="n">
@@ -52034,22 +52022,22 @@
       <c r="A805" s="27" t="n">
         <v>45693</v>
       </c>
-      <c r="B805" s="32" t="n">
+      <c r="B805" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="C805" s="33" t="n">
+      <c r="C805" s="32" t="n">
         <v>7</v>
       </c>
-      <c r="D805" s="33" t="n">
+      <c r="D805" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="E805" s="33" t="n">
+      <c r="E805" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="F805" s="33" t="n">
+      <c r="F805" s="32" t="n">
         <v>43</v>
       </c>
-      <c r="G805" s="33" t="n">
+      <c r="G805" s="32" t="n">
         <v>2</v>
       </c>
       <c r="H805" s="12" t="n">
@@ -52063,22 +52051,22 @@
       <c r="A806" s="27" t="n">
         <v>45696</v>
       </c>
-      <c r="B806" s="32" t="n">
+      <c r="B806" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="C806" s="33" t="n">
+      <c r="C806" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="D806" s="33" t="n">
+      <c r="D806" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="E806" s="33" t="n">
+      <c r="E806" s="32" t="n">
         <v>27</v>
       </c>
-      <c r="F806" s="33" t="n">
+      <c r="F806" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="G806" s="33" t="n">
+      <c r="G806" s="32" t="n">
         <v>9</v>
       </c>
       <c r="H806" s="12" t="n">
@@ -52092,22 +52080,22 @@
       <c r="A807" s="27" t="n">
         <v>45700</v>
       </c>
-      <c r="B807" s="32" t="n">
+      <c r="B807" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="C807" s="33" t="n">
+      <c r="C807" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="D807" s="33" t="n">
+      <c r="D807" s="32" t="n">
         <v>7</v>
       </c>
-      <c r="E807" s="33" t="n">
+      <c r="E807" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="F807" s="33" t="n">
+      <c r="F807" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="G807" s="33" t="n">
+      <c r="G807" s="32" t="n">
         <v>4</v>
       </c>
       <c r="H807" s="12" t="n">
@@ -52121,22 +52109,22 @@
       <c r="A808" s="27" t="n">
         <v>45703</v>
       </c>
-      <c r="B808" s="32" t="n">
+      <c r="B808" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="C808" s="33" t="n">
+      <c r="C808" s="32" t="n">
         <v>13</v>
       </c>
-      <c r="D808" s="33" t="n">
+      <c r="D808" s="32" t="n">
         <v>27</v>
       </c>
-      <c r="E808" s="33" t="n">
+      <c r="E808" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="F808" s="33" t="n">
+      <c r="F808" s="32" t="n">
         <v>41</v>
       </c>
-      <c r="G808" s="33" t="n">
+      <c r="G808" s="32" t="n">
         <v>10</v>
       </c>
       <c r="H808" s="12" t="n">
@@ -52150,22 +52138,22 @@
       <c r="A809" s="27" t="n">
         <v>45707</v>
       </c>
-      <c r="B809" s="32" t="n">
+      <c r="B809" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="C809" s="33" t="n">
+      <c r="C809" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="D809" s="33" t="n">
+      <c r="D809" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="E809" s="33" t="n">
+      <c r="E809" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="F809" s="33" t="n">
+      <c r="F809" s="32" t="n">
         <v>39</v>
       </c>
-      <c r="G809" s="33" t="n">
+      <c r="G809" s="32" t="n">
         <v>3</v>
       </c>
       <c r="H809" s="12" t="n">
@@ -52179,22 +52167,22 @@
       <c r="A810" s="27" t="n">
         <v>45710</v>
       </c>
-      <c r="B810" s="32" t="n">
+      <c r="B810" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="C810" s="33" t="n">
+      <c r="C810" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="D810" s="33" t="n">
+      <c r="D810" s="32" t="n">
         <v>19</v>
       </c>
-      <c r="E810" s="33" t="n">
+      <c r="E810" s="32" t="n">
         <v>33</v>
       </c>
-      <c r="F810" s="33" t="n">
+      <c r="F810" s="32" t="n">
         <v>38</v>
       </c>
-      <c r="G810" s="33" t="n">
+      <c r="G810" s="32" t="n">
         <v>8</v>
       </c>
       <c r="H810" s="12" t="n">
@@ -52208,22 +52196,22 @@
       <c r="A811" s="27" t="n">
         <v>45714</v>
       </c>
-      <c r="B811" s="32" t="n">
+      <c r="B811" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="C811" s="33" t="n">
+      <c r="C811" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="D811" s="33" t="n">
+      <c r="D811" s="32" t="n">
         <v>19</v>
       </c>
-      <c r="E811" s="33" t="n">
+      <c r="E811" s="32" t="n">
         <v>21</v>
       </c>
-      <c r="F811" s="33" t="n">
+      <c r="F811" s="32" t="n">
         <v>43</v>
       </c>
-      <c r="G811" s="33" t="n">
+      <c r="G811" s="32" t="n">
         <v>9</v>
       </c>
       <c r="H811" s="12" t="n">
@@ -52237,22 +52225,22 @@
       <c r="A812" s="27" t="n">
         <v>45717</v>
       </c>
-      <c r="B812" s="32" t="n">
+      <c r="B812" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="C812" s="33" t="n">
+      <c r="C812" s="32" t="n">
         <v>21</v>
       </c>
-      <c r="D812" s="33" t="n">
+      <c r="D812" s="32" t="n">
         <v>26</v>
       </c>
-      <c r="E812" s="33" t="n">
+      <c r="E812" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="F812" s="33" t="n">
+      <c r="F812" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="G812" s="33" t="n">
+      <c r="G812" s="32" t="n">
         <v>12</v>
       </c>
       <c r="H812" s="12" t="n">
@@ -52266,22 +52254,22 @@
       <c r="A813" s="27" t="n">
         <v>45721</v>
       </c>
-      <c r="B813" s="32" t="n">
+      <c r="B813" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="C813" s="33" t="n">
+      <c r="C813" s="32" t="n">
         <v>14</v>
       </c>
-      <c r="D813" s="33" t="n">
+      <c r="D813" s="32" t="n">
         <v>19</v>
       </c>
-      <c r="E813" s="33" t="n">
+      <c r="E813" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="F813" s="33" t="n">
+      <c r="F813" s="32" t="n">
         <v>43</v>
       </c>
-      <c r="G813" s="33" t="n">
+      <c r="G813" s="32" t="n">
         <v>6</v>
       </c>
       <c r="H813" s="12" t="n">
@@ -52295,22 +52283,22 @@
       <c r="A814" s="27" t="n">
         <v>45724</v>
       </c>
-      <c r="B814" s="32" t="n">
+      <c r="B814" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="C814" s="33" t="n">
+      <c r="C814" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="D814" s="33" t="n">
+      <c r="D814" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="E814" s="33" t="n">
+      <c r="E814" s="32" t="n">
         <v>33</v>
       </c>
-      <c r="F814" s="33" t="n">
+      <c r="F814" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="G814" s="33" t="n">
+      <c r="G814" s="32" t="n">
         <v>4</v>
       </c>
       <c r="H814" s="12" t="n">
@@ -52324,22 +52312,22 @@
       <c r="A815" s="27" t="n">
         <v>45728</v>
       </c>
-      <c r="B815" s="32" t="n">
+      <c r="B815" s="31" t="n">
         <v>17</v>
       </c>
-      <c r="C815" s="33" t="n">
+      <c r="C815" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="D815" s="33" t="n">
+      <c r="D815" s="32" t="n">
         <v>26</v>
       </c>
-      <c r="E815" s="33" t="n">
+      <c r="E815" s="32" t="n">
         <v>27</v>
       </c>
-      <c r="F815" s="33" t="n">
+      <c r="F815" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="G815" s="33" t="n">
+      <c r="G815" s="32" t="n">
         <v>1</v>
       </c>
       <c r="H815" s="12" t="n">
@@ -52353,22 +52341,22 @@
       <c r="A816" s="27" t="n">
         <v>45731</v>
       </c>
-      <c r="B816" s="32" t="n">
+      <c r="B816" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C816" s="33" t="n">
+      <c r="C816" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="D816" s="33" t="n">
+      <c r="D816" s="32" t="n">
         <v>13</v>
       </c>
-      <c r="E816" s="33" t="n">
+      <c r="E816" s="32" t="n">
         <v>31</v>
       </c>
-      <c r="F816" s="33" t="n">
+      <c r="F816" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="G816" s="33" t="n">
+      <c r="G816" s="32" t="n">
         <v>16</v>
       </c>
       <c r="H816" s="12" t="n">
@@ -52382,22 +52370,22 @@
       <c r="A817" s="27" t="n">
         <v>45735</v>
       </c>
-      <c r="B817" s="32" t="n">
+      <c r="B817" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="C817" s="33" t="n">
+      <c r="C817" s="32" t="n">
         <v>15</v>
       </c>
-      <c r="D817" s="33" t="n">
+      <c r="D817" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="E817" s="33" t="n">
+      <c r="E817" s="32" t="n">
         <v>28</v>
       </c>
-      <c r="F817" s="33" t="n">
+      <c r="F817" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="G817" s="33" t="n">
+      <c r="G817" s="32" t="n">
         <v>11</v>
       </c>
       <c r="H817" s="12" t="n">
@@ -52411,22 +52399,22 @@
       <c r="A818" s="27" t="n">
         <v>45738</v>
       </c>
-      <c r="B818" s="32" t="n">
+      <c r="B818" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="C818" s="33" t="n">
+      <c r="C818" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="D818" s="33" t="n">
+      <c r="D818" s="32" t="n">
         <v>17</v>
       </c>
-      <c r="E818" s="33" t="n">
+      <c r="E818" s="32" t="n">
         <v>31</v>
       </c>
-      <c r="F818" s="33" t="n">
+      <c r="F818" s="32" t="n">
         <v>40</v>
       </c>
-      <c r="G818" s="33" t="n">
+      <c r="G818" s="32" t="n">
         <v>16</v>
       </c>
       <c r="H818" s="12" t="n">
@@ -52440,22 +52428,22 @@
       <c r="A819" s="27" t="n">
         <v>45742</v>
       </c>
-      <c r="B819" s="32" t="n">
+      <c r="B819" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="C819" s="33" t="n">
+      <c r="C819" s="32" t="n">
         <v>13</v>
       </c>
-      <c r="D819" s="33" t="n">
+      <c r="D819" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="E819" s="33" t="n">
+      <c r="E819" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="F819" s="33" t="n">
+      <c r="F819" s="32" t="n">
         <v>43</v>
       </c>
-      <c r="G819" s="33" t="n">
+      <c r="G819" s="32" t="n">
         <v>2</v>
       </c>
       <c r="H819" s="12" t="n">
@@ -52469,22 +52457,22 @@
       <c r="A820" s="27" t="n">
         <v>45745</v>
       </c>
-      <c r="B820" s="32" t="n">
+      <c r="B820" s="31" t="n">
         <v>17</v>
       </c>
-      <c r="C820" s="33" t="n">
+      <c r="C820" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="D820" s="33" t="n">
+      <c r="D820" s="32" t="n">
         <v>27</v>
       </c>
-      <c r="E820" s="33" t="n">
+      <c r="E820" s="32" t="n">
         <v>28</v>
       </c>
-      <c r="F820" s="33" t="n">
+      <c r="F820" s="32" t="n">
         <v>39</v>
       </c>
-      <c r="G820" s="33" t="n">
+      <c r="G820" s="32" t="n">
         <v>3</v>
       </c>
       <c r="H820" s="12" t="n">
@@ -52498,22 +52486,22 @@
       <c r="A821" s="27" t="n">
         <v>45749</v>
       </c>
-      <c r="B821" s="32" t="n">
+      <c r="B821" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="C821" s="33" t="n">
+      <c r="C821" s="32" t="n">
         <v>13</v>
       </c>
-      <c r="D821" s="33" t="n">
+      <c r="D821" s="32" t="n">
         <v>20</v>
       </c>
-      <c r="E821" s="33" t="n">
+      <c r="E821" s="32" t="n">
         <v>23</v>
       </c>
-      <c r="F821" s="33" t="n">
+      <c r="F821" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="G821" s="33" t="n">
+      <c r="G821" s="32" t="n">
         <v>10</v>
       </c>
       <c r="H821" s="12" t="n">
@@ -52527,22 +52515,22 @@
       <c r="A822" s="27" t="n">
         <v>45752</v>
       </c>
-      <c r="B822" s="32" t="n">
+      <c r="B822" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="C822" s="33" t="n">
+      <c r="C822" s="32" t="n">
         <v>9</v>
       </c>
-      <c r="D822" s="33" t="n">
+      <c r="D822" s="32" t="n">
         <v>17</v>
       </c>
-      <c r="E822" s="33" t="n">
+      <c r="E822" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="F822" s="33" t="n">
+      <c r="F822" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="G822" s="33" t="n">
+      <c r="G822" s="32" t="n">
         <v>5</v>
       </c>
       <c r="H822" s="12" t="n">
@@ -52556,22 +52544,22 @@
       <c r="A823" s="27" t="n">
         <v>45756</v>
       </c>
-      <c r="B823" s="32" t="n">
+      <c r="B823" s="31" t="n">
         <v>12</v>
       </c>
-      <c r="C823" s="33" t="n">
+      <c r="C823" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="D823" s="33" t="n">
+      <c r="D823" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="E823" s="33" t="n">
+      <c r="E823" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="F823" s="33" t="n">
+      <c r="F823" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="G823" s="33" t="n">
+      <c r="G823" s="32" t="n">
         <v>9</v>
       </c>
       <c r="H823" s="12" t="n">
@@ -52585,22 +52573,22 @@
       <c r="A824" s="27" t="n">
         <v>45759</v>
       </c>
-      <c r="B824" s="32" t="n">
+      <c r="B824" s="31" t="n">
         <v>21</v>
       </c>
-      <c r="C824" s="33" t="n">
+      <c r="C824" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="D824" s="33" t="n">
+      <c r="D824" s="32" t="n">
         <v>38</v>
       </c>
-      <c r="E824" s="33" t="n">
+      <c r="E824" s="32" t="n">
         <v>39</v>
       </c>
-      <c r="F824" s="33" t="n">
+      <c r="F824" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="G824" s="33" t="n">
+      <c r="G824" s="32" t="n">
         <v>15</v>
       </c>
       <c r="H824" s="12" t="n">
@@ -52614,22 +52602,22 @@
       <c r="A825" s="27" t="n">
         <v>45763</v>
       </c>
-      <c r="B825" s="32" t="n">
+      <c r="B825" s="31" t="n">
         <v>18</v>
       </c>
-      <c r="C825" s="33" t="n">
+      <c r="C825" s="32" t="n">
         <v>32</v>
       </c>
-      <c r="D825" s="33" t="n">
+      <c r="D825" s="32" t="n">
         <v>34</v>
       </c>
-      <c r="E825" s="33" t="n">
+      <c r="E825" s="32" t="n">
         <v>36</v>
       </c>
-      <c r="F825" s="33" t="n">
+      <c r="F825" s="32" t="n">
         <v>38</v>
       </c>
-      <c r="G825" s="33" t="n">
+      <c r="G825" s="32" t="n">
         <v>13</v>
       </c>
       <c r="H825" s="12" t="n">

</xml_diff>

<commit_message>
chore: update baloto.xlsx with latest draw results
</commit_message>
<xml_diff>
--- a/baloto.xlsx
+++ b/baloto.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I961"/>
+  <dimension ref="A1:I963"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="10.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -28337,6 +28337,64 @@
         <v>0</v>
       </c>
     </row>
+    <row r="962">
+      <c r="A962" s="3" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B962" t="n">
+        <v>3</v>
+      </c>
+      <c r="C962" t="n">
+        <v>5</v>
+      </c>
+      <c r="D962" t="n">
+        <v>13</v>
+      </c>
+      <c r="E962" t="n">
+        <v>15</v>
+      </c>
+      <c r="F962" t="n">
+        <v>25</v>
+      </c>
+      <c r="G962" t="n">
+        <v>9</v>
+      </c>
+      <c r="H962" t="n">
+        <v>0</v>
+      </c>
+      <c r="I962" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="3" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B963" t="n">
+        <v>1</v>
+      </c>
+      <c r="C963" t="n">
+        <v>8</v>
+      </c>
+      <c r="D963" t="n">
+        <v>17</v>
+      </c>
+      <c r="E963" t="n">
+        <v>19</v>
+      </c>
+      <c r="F963" t="n">
+        <v>40</v>
+      </c>
+      <c r="G963" t="n">
+        <v>10</v>
+      </c>
+      <c r="H963" t="n">
+        <v>0</v>
+      </c>
+      <c r="I963" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28348,7 +28406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I947"/>
+  <dimension ref="A1:I949"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="10.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -55837,6 +55895,64 @@
         <v>0</v>
       </c>
     </row>
+    <row r="948">
+      <c r="A948" s="3" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B948" t="n">
+        <v>9</v>
+      </c>
+      <c r="C948" t="n">
+        <v>24</v>
+      </c>
+      <c r="D948" t="n">
+        <v>25</v>
+      </c>
+      <c r="E948" t="n">
+        <v>29</v>
+      </c>
+      <c r="F948" t="n">
+        <v>42</v>
+      </c>
+      <c r="G948" t="n">
+        <v>2</v>
+      </c>
+      <c r="H948" t="n">
+        <v>0</v>
+      </c>
+      <c r="I948" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="3" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B949" t="n">
+        <v>1</v>
+      </c>
+      <c r="C949" t="n">
+        <v>2</v>
+      </c>
+      <c r="D949" t="n">
+        <v>13</v>
+      </c>
+      <c r="E949" t="n">
+        <v>19</v>
+      </c>
+      <c r="F949" t="n">
+        <v>43</v>
+      </c>
+      <c r="G949" t="n">
+        <v>6</v>
+      </c>
+      <c r="H949" t="n">
+        <v>0</v>
+      </c>
+      <c r="I949" t="n">
+        <v>22244250</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update baloto.xlsx with latest draw data
</commit_message>
<xml_diff>
--- a/baloto.xlsx
+++ b/baloto.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I963"/>
+  <dimension ref="A1:I966"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="10.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -28395,6 +28395,93 @@
         <v>0</v>
       </c>
     </row>
+    <row r="964">
+      <c r="A964" s="3" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B964" t="n">
+        <v>1</v>
+      </c>
+      <c r="C964" t="n">
+        <v>12</v>
+      </c>
+      <c r="D964" t="n">
+        <v>13</v>
+      </c>
+      <c r="E964" t="n">
+        <v>34</v>
+      </c>
+      <c r="F964" t="n">
+        <v>35</v>
+      </c>
+      <c r="G964" t="n">
+        <v>15</v>
+      </c>
+      <c r="H964" t="n">
+        <v>0</v>
+      </c>
+      <c r="I964" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="3" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B965" t="n">
+        <v>4</v>
+      </c>
+      <c r="C965" t="n">
+        <v>19</v>
+      </c>
+      <c r="D965" t="n">
+        <v>31</v>
+      </c>
+      <c r="E965" t="n">
+        <v>38</v>
+      </c>
+      <c r="F965" t="n">
+        <v>39</v>
+      </c>
+      <c r="G965" t="n">
+        <v>4</v>
+      </c>
+      <c r="H965" t="n">
+        <v>0</v>
+      </c>
+      <c r="I965" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="3" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B966" t="n">
+        <v>7</v>
+      </c>
+      <c r="C966" t="n">
+        <v>21</v>
+      </c>
+      <c r="D966" t="n">
+        <v>25</v>
+      </c>
+      <c r="E966" t="n">
+        <v>40</v>
+      </c>
+      <c r="F966" t="n">
+        <v>43</v>
+      </c>
+      <c r="G966" t="n">
+        <v>11</v>
+      </c>
+      <c r="H966" t="n">
+        <v>0</v>
+      </c>
+      <c r="I966" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28406,7 +28493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I949"/>
+  <dimension ref="A1:I952"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="10.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -55953,6 +56040,93 @@
         <v>22244250</v>
       </c>
     </row>
+    <row r="950">
+      <c r="A950" s="3" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B950" t="n">
+        <v>6</v>
+      </c>
+      <c r="C950" t="n">
+        <v>12</v>
+      </c>
+      <c r="D950" t="n">
+        <v>15</v>
+      </c>
+      <c r="E950" t="n">
+        <v>23</v>
+      </c>
+      <c r="F950" t="n">
+        <v>31</v>
+      </c>
+      <c r="G950" t="n">
+        <v>16</v>
+      </c>
+      <c r="H950" t="n">
+        <v>0</v>
+      </c>
+      <c r="I950" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="3" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B951" t="n">
+        <v>3</v>
+      </c>
+      <c r="C951" t="n">
+        <v>15</v>
+      </c>
+      <c r="D951" t="n">
+        <v>16</v>
+      </c>
+      <c r="E951" t="n">
+        <v>22</v>
+      </c>
+      <c r="F951" t="n">
+        <v>38</v>
+      </c>
+      <c r="G951" t="n">
+        <v>2</v>
+      </c>
+      <c r="H951" t="n">
+        <v>0</v>
+      </c>
+      <c r="I951" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="3" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B952" t="n">
+        <v>4</v>
+      </c>
+      <c r="C952" t="n">
+        <v>9</v>
+      </c>
+      <c r="D952" t="n">
+        <v>16</v>
+      </c>
+      <c r="E952" t="n">
+        <v>22</v>
+      </c>
+      <c r="F952" t="n">
+        <v>28</v>
+      </c>
+      <c r="G952" t="n">
+        <v>15</v>
+      </c>
+      <c r="H952" t="n">
+        <v>0</v>
+      </c>
+      <c r="I952" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: standardize execution paths and use local virtual environment python interpreter across shell scripts
</commit_message>
<xml_diff>
--- a/baloto.xlsx
+++ b/baloto.xlsx
@@ -28514,28 +28514,28 @@
       <c r="A970" s="8" t="n">
         <v>46167</v>
       </c>
-      <c r="B970" t="n">
+      <c r="B970" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C970" t="n">
+      <c r="C970" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="D970" t="n">
+      <c r="D970" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="E970" t="n">
+      <c r="E970" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="F970" t="n">
+      <c r="F970" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="G970" t="n">
+      <c r="G970" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="H970" t="n">
-        <v>0</v>
-      </c>
-      <c r="I970" t="n">
+      <c r="H970" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I970" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28543,29 +28543,145 @@
       <c r="A971" s="8" t="n">
         <v>46169</v>
       </c>
-      <c r="B971" t="n">
+      <c r="B971" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C971" t="n">
+      <c r="C971" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="D971" t="n">
+      <c r="D971" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="E971" t="n">
+      <c r="E971" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="F971" t="n">
+      <c r="F971" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="G971" t="n">
+      <c r="G971" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="H971" t="n">
-        <v>0</v>
-      </c>
-      <c r="I971" t="n">
+      <c r="H971" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I971" s="4" t="n">
         <v>37693100</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="8" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B972" t="n">
+        <v>26</v>
+      </c>
+      <c r="C972" t="n">
+        <v>29</v>
+      </c>
+      <c r="D972" t="n">
+        <v>35</v>
+      </c>
+      <c r="E972" t="n">
+        <v>38</v>
+      </c>
+      <c r="F972" t="n">
+        <v>41</v>
+      </c>
+      <c r="G972" t="n">
+        <v>11</v>
+      </c>
+      <c r="H972" t="n">
+        <v>0</v>
+      </c>
+      <c r="I972" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="8" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B973" t="n">
+        <v>5</v>
+      </c>
+      <c r="C973" t="n">
+        <v>15</v>
+      </c>
+      <c r="D973" t="n">
+        <v>19</v>
+      </c>
+      <c r="E973" t="n">
+        <v>28</v>
+      </c>
+      <c r="F973" t="n">
+        <v>32</v>
+      </c>
+      <c r="G973" t="n">
+        <v>1</v>
+      </c>
+      <c r="H973" t="n">
+        <v>0</v>
+      </c>
+      <c r="I973" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="8" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B974" t="n">
+        <v>6</v>
+      </c>
+      <c r="C974" t="n">
+        <v>8</v>
+      </c>
+      <c r="D974" t="n">
+        <v>9</v>
+      </c>
+      <c r="E974" t="n">
+        <v>32</v>
+      </c>
+      <c r="F974" t="n">
+        <v>40</v>
+      </c>
+      <c r="G974" t="n">
+        <v>13</v>
+      </c>
+      <c r="H974" t="n">
+        <v>0</v>
+      </c>
+      <c r="I974" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="8" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B975" t="n">
+        <v>3</v>
+      </c>
+      <c r="C975" t="n">
+        <v>5</v>
+      </c>
+      <c r="D975" t="n">
+        <v>17</v>
+      </c>
+      <c r="E975" t="n">
+        <v>18</v>
+      </c>
+      <c r="F975" t="n">
+        <v>27</v>
+      </c>
+      <c r="G975" t="n">
+        <v>7</v>
+      </c>
+      <c r="H975" t="n">
+        <v>0</v>
+      </c>
+      <c r="I975" t="n">
+        <v>38507200</v>
       </c>
     </row>
     <row r="976" ht="15" customHeight="1" s="5">
@@ -28584,7 +28700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I957"/>
+  <dimension ref="A1:I961"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10.71" customWidth="1" style="4" min="1" max="1"/>
@@ -56309,28 +56425,28 @@
       <c r="A956" s="8" t="n">
         <v>46167</v>
       </c>
-      <c r="B956" t="n">
+      <c r="B956" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C956" t="n">
+      <c r="C956" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="D956" t="n">
+      <c r="D956" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="E956" t="n">
+      <c r="E956" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="F956" t="n">
+      <c r="F956" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="G956" t="n">
+      <c r="G956" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="H956" t="n">
-        <v>0</v>
-      </c>
-      <c r="I956" t="n">
+      <c r="H956" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I956" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -56338,29 +56454,145 @@
       <c r="A957" s="8" t="n">
         <v>46169</v>
       </c>
-      <c r="B957" t="n">
+      <c r="B957" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C957" t="n">
+      <c r="C957" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="D957" t="n">
+      <c r="D957" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="E957" t="n">
+      <c r="E957" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="F957" t="n">
+      <c r="F957" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="G957" t="n">
+      <c r="G957" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="H957" t="n">
-        <v>0</v>
-      </c>
-      <c r="I957" t="n">
-        <v>0</v>
+      <c r="H957" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I957" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="8" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B958" t="n">
+        <v>4</v>
+      </c>
+      <c r="C958" t="n">
+        <v>12</v>
+      </c>
+      <c r="D958" t="n">
+        <v>13</v>
+      </c>
+      <c r="E958" t="n">
+        <v>31</v>
+      </c>
+      <c r="F958" t="n">
+        <v>35</v>
+      </c>
+      <c r="G958" t="n">
+        <v>9</v>
+      </c>
+      <c r="H958" t="n">
+        <v>0</v>
+      </c>
+      <c r="I958" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="8" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B959" t="n">
+        <v>7</v>
+      </c>
+      <c r="C959" t="n">
+        <v>11</v>
+      </c>
+      <c r="D959" t="n">
+        <v>25</v>
+      </c>
+      <c r="E959" t="n">
+        <v>32</v>
+      </c>
+      <c r="F959" t="n">
+        <v>36</v>
+      </c>
+      <c r="G959" t="n">
+        <v>8</v>
+      </c>
+      <c r="H959" t="n">
+        <v>0</v>
+      </c>
+      <c r="I959" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="8" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B960" t="n">
+        <v>14</v>
+      </c>
+      <c r="C960" t="n">
+        <v>26</v>
+      </c>
+      <c r="D960" t="n">
+        <v>30</v>
+      </c>
+      <c r="E960" t="n">
+        <v>37</v>
+      </c>
+      <c r="F960" t="n">
+        <v>39</v>
+      </c>
+      <c r="G960" t="n">
+        <v>2</v>
+      </c>
+      <c r="H960" t="n">
+        <v>0</v>
+      </c>
+      <c r="I960" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="8" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B961" t="n">
+        <v>7</v>
+      </c>
+      <c r="C961" t="n">
+        <v>14</v>
+      </c>
+      <c r="D961" t="n">
+        <v>22</v>
+      </c>
+      <c r="E961" t="n">
+        <v>35</v>
+      </c>
+      <c r="F961" t="n">
+        <v>41</v>
+      </c>
+      <c r="G961" t="n">
+        <v>6</v>
+      </c>
+      <c r="H961" t="n">
+        <v>0</v>
+      </c>
+      <c r="I961" t="n">
+        <v>17492400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add web launcher and implement categorical scoring thresholds for JAX analysis in Streamlit app
</commit_message>
<xml_diff>
--- a/baloto.xlsx
+++ b/baloto.xlsx
@@ -17,10 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -28572,28 +28571,28 @@
       <c r="A972" s="8" t="n">
         <v>46176</v>
       </c>
-      <c r="B972" t="n">
+      <c r="B972" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="C972" t="n">
+      <c r="C972" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="D972" t="n">
+      <c r="D972" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="E972" t="n">
+      <c r="E972" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="F972" t="n">
+      <c r="F972" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="G972" t="n">
+      <c r="G972" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="H972" t="n">
-        <v>0</v>
-      </c>
-      <c r="I972" t="n">
+      <c r="H972" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I972" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28601,28 +28600,28 @@
       <c r="A973" s="8" t="n">
         <v>46179</v>
       </c>
-      <c r="B973" t="n">
+      <c r="B973" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C973" t="n">
+      <c r="C973" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="D973" t="n">
+      <c r="D973" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="E973" t="n">
+      <c r="E973" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="F973" t="n">
+      <c r="F973" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="G973" t="n">
+      <c r="G973" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H973" t="n">
-        <v>0</v>
-      </c>
-      <c r="I973" t="n">
+      <c r="H973" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I973" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28630,28 +28629,28 @@
       <c r="A974" s="8" t="n">
         <v>46181</v>
       </c>
-      <c r="B974" t="n">
+      <c r="B974" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C974" t="n">
+      <c r="C974" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="D974" t="n">
+      <c r="D974" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="E974" t="n">
+      <c r="E974" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="F974" t="n">
+      <c r="F974" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="G974" t="n">
+      <c r="G974" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="H974" t="n">
-        <v>0</v>
-      </c>
-      <c r="I974" t="n">
+      <c r="H974" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I974" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -28659,28 +28658,28 @@
       <c r="A975" s="8" t="n">
         <v>46183</v>
       </c>
-      <c r="B975" t="n">
+      <c r="B975" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C975" t="n">
+      <c r="C975" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D975" t="n">
+      <c r="D975" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="E975" t="n">
+      <c r="E975" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="F975" t="n">
+      <c r="F975" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="G975" t="n">
+      <c r="G975" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H975" t="n">
-        <v>0</v>
-      </c>
-      <c r="I975" t="n">
+      <c r="H975" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I975" s="4" t="n">
         <v>38507200</v>
       </c>
     </row>
@@ -56483,28 +56482,28 @@
       <c r="A958" s="8" t="n">
         <v>46176</v>
       </c>
-      <c r="B958" t="n">
+      <c r="B958" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C958" t="n">
+      <c r="C958" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="D958" t="n">
+      <c r="D958" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="E958" t="n">
+      <c r="E958" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="F958" t="n">
+      <c r="F958" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="G958" t="n">
+      <c r="G958" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H958" t="n">
-        <v>0</v>
-      </c>
-      <c r="I958" t="n">
+      <c r="H958" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I958" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -56512,28 +56511,28 @@
       <c r="A959" s="8" t="n">
         <v>46179</v>
       </c>
-      <c r="B959" t="n">
+      <c r="B959" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C959" t="n">
+      <c r="C959" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="D959" t="n">
+      <c r="D959" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="E959" t="n">
+      <c r="E959" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="F959" t="n">
+      <c r="F959" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="G959" t="n">
+      <c r="G959" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="H959" t="n">
-        <v>0</v>
-      </c>
-      <c r="I959" t="n">
+      <c r="H959" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I959" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -56541,28 +56540,28 @@
       <c r="A960" s="8" t="n">
         <v>46181</v>
       </c>
-      <c r="B960" t="n">
+      <c r="B960" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="C960" t="n">
+      <c r="C960" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="D960" t="n">
+      <c r="D960" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="E960" t="n">
+      <c r="E960" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="F960" t="n">
+      <c r="F960" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="G960" t="n">
+      <c r="G960" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H960" t="n">
-        <v>0</v>
-      </c>
-      <c r="I960" t="n">
+      <c r="H960" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I960" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -56570,28 +56569,28 @@
       <c r="A961" s="8" t="n">
         <v>46183</v>
       </c>
-      <c r="B961" t="n">
+      <c r="B961" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C961" t="n">
+      <c r="C961" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="D961" t="n">
+      <c r="D961" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="E961" t="n">
+      <c r="E961" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="F961" t="n">
+      <c r="F961" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="G961" t="n">
+      <c r="G961" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H961" t="n">
-        <v>0</v>
-      </c>
-      <c r="I961" t="n">
+      <c r="H961" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I961" s="4" t="n">
         <v>17492400</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor installation script and update requirements
- Updated `instalar.bat` for improved readability and consistency.
- Ensured Python version check and UV installation process are clear.
- Added feedback for existing virtual environment and dependencies installation.
- Cleaned up `requirements.txt` formatting for better clarity.
- Minor formatting adjustments in `debug_scraping.py` for consistency.
</commit_message>
<xml_diff>
--- a/baloto.xlsx
+++ b/baloto.xlsx
@@ -26484,16 +26484,16 @@
         <v>45966</v>
       </c>
       <c r="B900" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C900" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="D900" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E900" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="C900" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="D900" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="E900" s="4" t="n">
-        <v>35</v>
       </c>
       <c r="F900" s="4" t="n">
         <v>40</v>
@@ -26513,16 +26513,16 @@
         <v>45966</v>
       </c>
       <c r="B901" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C901" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="C901" s="4" t="n">
+      <c r="D901" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="D901" s="4" t="n">
+      <c r="E901" s="4" t="n">
         <v>35</v>
-      </c>
-      <c r="E901" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="F901" s="4" t="n">
         <v>40</v>
@@ -28684,7 +28684,33 @@
       </c>
     </row>
     <row r="976" ht="15" customHeight="1" s="5">
-      <c r="F976" s="9" t="n"/>
+      <c r="A976" s="8" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B976" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C976" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D976" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="E976" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="F976" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="G976" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H976" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I976" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -28699,7 +28725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I961"/>
+  <dimension ref="A1:I962"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10.71" customWidth="1" style="4" min="1" max="1"/>
@@ -56594,6 +56620,35 @@
         <v>17492400</v>
       </c>
     </row>
+    <row r="962">
+      <c r="A962" s="8" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B962" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="C962" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="D962" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="E962" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="F962" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="G962" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H962" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I962" s="4" t="n">
+        <v>24189500</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>